<commit_message>
updated discourse annotation ted-mdb 1971
</commit_message>
<xml_diff>
--- a/annotators/team/tg/de/annotated/ted-mdb.1971.xlsx
+++ b/annotators/team/tg/de/annotated/ted-mdb.1971.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\de\in-progress\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\de\annotated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8426F333-07E5-4064-A209-9195F3E2E862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD172854-9236-4B37-9129-63F51D6BCDF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="15204" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sentence-level annotation" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1399" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1399" uniqueCount="502">
   <si>
     <t>ID</t>
   </si>
@@ -1524,6 +1524,9 @@
   </si>
   <si>
     <t>NoRel, weil kein einzelner Satz (deiktisch) zuzuordnen?</t>
+  </si>
+  <si>
+    <t>(weil)</t>
   </si>
 </sst>
 </file>
@@ -2480,13 +2483,13 @@
         <v>11</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>473</v>
+        <v>501</v>
       </c>
       <c r="H15" s="10">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="J15" s="12" t="s">
         <v>499</v>

</xml_diff>